<commit_message>
feat(F-NAR-019): ATOM-AUT.ROU.001-08 Le chocolat de Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.ROU.001-08.xlsx
+++ b/stories/arbres/ATOM-AUT.ROU.001-08.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina sent le cacao et veut le bol tout de suite. La casserole chante encore. Une chose puis la suivante, elle souffle, boit, et une moustache brune apparaît.</t>
+          <t>Le radiateur fait tic. Une chaussette brune y respire. Un anneau de vapeur glisse sous la porte. Sur le bord, un éclat de casserole brille. Nina veut le chocolat maintenant. Elle saisit le bol : trop chaud, une goutte tombe. Elle refuse de foncer, chaussettes, bol sur le chariot. Les roues tournent. Près du radiateur, l'éclat tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La maison sent déjà le cacao. Dans la cuisine, une casserole chante. Elle fait des petites bulles. Une vapeur glisse sous la porte. Elle est tiède. Elle sent le sucre. Elle sent aussi le lait chaud. La vapeur chatouille un peu le nez. Nina, tu sens le chocolat ? Oui, maman. C'est bon. Il n'est pas encore dans le bol. Près du radiateur, des chaussettes sèchent. Elles sont épaisses et brunes. En ce moment, Nina ouvre les yeux. Je veux le chocolat. Nina va vers la cuisine. Elle est encore en pyjama. La casserole chante encore. Il finit de se faire. D'abord le pull. Une chose, puis la suivante. Nina s'arrête près du radiateur. Elle touche une chaussette. La chaussette est tiède. On se lève ? Oui. Nina revient vers le lit. Ses pieds touchent le tapis. Le tapis est doux. Le pull, maintenant.</t>
+          <t>Le radiateur fait tic, près du lit. Une chaussette brune y respire. Elle est épaisse, un peu rêche. L'air sent le lait chaud. Sous la porte, un anneau de vapeur glisse. Il chatouille un peu le nez. Nina, tu sens le chocolat ? Oui, maman. Je le veux maintenant ! Dans la cuisine, une casserole chante. Elle fait de petites bulles. Sur le bord, un éclat de casserole brille. Il est blanc, papa. C'est le lait, sur le métal. Près de la table, un petit chariot attend. Ses deux roues sont en bois. Le bois est lisse, un peu clair. Le pyjama de Nina est chaud. Le tapis tient ses pieds. Le bol n'est pas sur la table. En ce moment, Nina saute du lit. Ses pieds trouvent le tapis. J'y vais ! Elle court vers la cuisine, en pyjama. Le carrelage pique ses pieds. Le bol ! Nina saisit le bol d'un coup. Le bol brûle ses doigts. Elle le lâche. Une goutte brune tombe. Aïe. Le sourire de Nina disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes le chariot ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La maison sent déjà le cacao. Dans la cuisine, une casserole chante. Elle fait des petites bulles. Une vapeur glisse sous la porte. Elle est tiède. Elle sent le sucre. Elle sent aussi le lait chaud. La vapeur chatouille un peu le nez. Nina, tu sens le chocolat ? Oui, maman. C'est bon. Il n'est pas encore dans le bol. Près du radiateur, des chaussettes sèchent. Elles sont épaisses et brunes. En ce moment, Nina ouvre les yeux. Je veux le chocolat. Nina va vers la cuisine. Elle est encore en pyjama. La casserole chante encore. Il finit de se faire. D'abord le pull. Une chose, puis la suivante. Nina s'arrête près du radiateur. Elle touche une chaussette. La chaussette est tiède. On se lève ? Oui. Nina revient vers le lit. Ses pieds touchent le tapis. Le tapis est doux. Le pull, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le radiateur fait tic, près du lit. Une chaussette brune y respire. Elle est épaisse, un peu rêche. L'air sent le lait chaud. Sous la porte, un anneau de vapeur glisse. Il chatouille un peu le nez. Nina, tu sens le chocolat ? Oui, maman. Je le veux maintenant ! Dans la cuisine, une casserole chante. Elle fait de petites bulles. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de casserole&lt;/emphasis&gt; brille. Il est blanc, papa. C'est le lait, sur le métal. Près de la table, un petit chariot attend. Ses deux roues sont en bois. Le bois est lisse, un peu clair. Le pyjama de Nina est chaud. Le tapis tient ses pieds. Le bol n'est pas sur la table. En ce moment, Nina saute du lit. Ses pieds trouvent le tapis. J'y vais ! Elle court vers la cuisine, en pyjama. Le carrelage pique ses pieds. Le bol ! Nina saisit le bol d'un coup. Le bol brûle ses doigts. Elle le lâche. Une goutte brune tombe. Aïe. Le sourire de Nina disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes le chariot ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le soleil entre. Fabrice ouvre les yeux. Le drap est chaud. Papa dit : c'est le matin. &lt;emphasis&gt;une&lt;/emphasis&gt; étape après l'autre. D'abord, Fabrice se lève. Ses pieds touchent le tapis. Le tapis est doux. Ensuite, Fabrice s'habille. Il met le pull bleu. Il met le pantalon. Maman dit : maintenant, le déjeuner. Fabrice s'assoit à table. Il mange une compote. Il boit du lait tiède. Papa dit : ensuite, le sac. Fabrice met le cahier dans le sac. Fabrice met la gourde dans le sac. Chaque étape est finie. Fabrice est prêt. Papa dit : une étape après l'autre. C'est plus calme.&lt;/slow&gt; [pause]</t>
+          <t>Le radiateur fait tic, près du lit. Une chaussette brune y respire. Elle est épaisse, un peu rêche. L'air sent le lait chaud. Sous la porte, un anneau de vapeur glisse. Il chatouille un peu le nez. Nina, tu sens le chocolat ? Oui, maman. Je le veux maintenant ! Dans la cuisine, une casserole chante. Elle fait de petites bulles. Sur le bord, un &lt;emphasis&gt;éclat de casserole&lt;/emphasis&gt; brille. Il est blanc, papa. C'est le lait, sur le métal. Près de la table, un petit chariot attend. Ses deux roues sont en bois. Le bois est lisse, un peu clair. Le pyjama de Nina est chaud. Le tapis tient ses pieds. Le bol n'est pas sur la table. En ce moment, Nina saute du lit. Ses pieds trouvent le tapis. J'y vais ! Elle court vers la cuisine, en pyjama. Le carrelage pique ses pieds. Le bol ! Nina saisit le bol d'un coup. Le bol brûle ses doigts. Elle le lâche. Une goutte brune tombe. Aïe. Le sourire de Nina disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes le chariot ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>éclat de casserole</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,42 +1319,52 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_chocolat_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La maison sent déjà le cacao.
-narrateur|Dans la cuisine, une casserole chante.
-narrateur|Elle fait des petites bulles.
-narrateur|Une vapeur glisse sous la porte.
-narrateur|Elle est tiède.
-narrateur|Elle sent le sucre.
-narrateur|Elle sent aussi le lait chaud.
-narrateur|La vapeur chatouille un peu le nez.
+          <t>narrateur|Le radiateur fait tic, près du lit.
+narrateur|Une chaussette brune y respire.
+narrateur|Elle est épaisse, un peu rêche.
+narrateur|L'air sent le lait chaud.
+narrateur|Sous la porte, un anneau de vapeur glisse.
+narrateur|Il chatouille un peu le nez.
 maman|Nina, tu sens le chocolat ?
 enfant-f|Oui, maman.
-enfant-f|C'est bon.
-papa|Il n'est pas encore dans le bol.
-narrateur|Près du radiateur, des chaussettes sèchent.
-narrateur|Elles sont épaisses et brunes.
-narrateur|En ce moment, Nina ouvre les yeux.
-enfant-f|Je veux le chocolat.
-narrateur|Nina va vers la cuisine.
-narrateur|Elle est encore en pyjama.
-narrateur|La casserole chante encore.
-maman|Il finit de se faire.
-papa|D'abord le pull.
-papa|Une chose, puis la suivante.
-narrateur|Nina s'arrête près du radiateur.
-narrateur|Elle touche une chaussette.
-narrateur|La chaussette est tiède.
-maman|On se lève ?
-enfant-f|Oui.
-narrateur|Nina revient vers le lit.
-narrateur|Ses pieds touchent le tapis.
-narrateur|Le tapis est doux.
-maman|Le pull, maintenant.</t>
+enfant-f|Je le veux maintenant !
+narrateur|Dans la cuisine, une casserole chante.
+narrateur|Elle fait de petites bulles.
+narrateur|Sur le bord, un éclat de casserole brille.
+enfant-f|Il est blanc, papa.
+papa|C'est le lait, sur le métal.
+narrateur|Près de la table, un petit chariot attend.
+narrateur|Ses deux roues sont en bois.
+narrateur|Le bois est lisse, un peu clair.
+narrateur|Le pyjama de Nina est chaud.
+narrateur|Le tapis tient ses pieds.
+papa|Le bol n'est pas sur la table.
+narrateur|En ce moment, Nina saute du lit.
+narrateur|Ses pieds trouvent le tapis.
+enfant-f|J'y vais !
+narrateur|Elle court vers la cuisine, en pyjama.
+narrateur|Le carrelage pique ses pieds.
+enfant-f|Le bol !
+narrateur|Nina saisit le bol d'un coup.
+narrateur|Le bol brûle ses doigts.
+narrateur|Elle le lâche.
+narrateur|Une goutte brune tombe.
+enfant-f|Aïe.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes le chariot ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1386,27 +1396,27 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Nina veut le chocolat. Comment se prépare-t-elle ?</t>
+          <t>Nina veut le chocolat. Comment le bol avance-t-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nina veut le chocolat. Comment se prépare-t-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina veut le chocolat. Comment le &lt;emphasis level="moderate"&gt;bol&lt;/emphasis&gt; avance-t-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Fabrice se prépare. Comment avance-t-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina veut le chocolat. Comment le &lt;emphasis&gt;bol&lt;/emphasis&gt; avance-t-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>une chose</t>
+          <t>il roule</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>une chose | puis l'autre | d'abord | doucement | une chose puis l'autre | puis la suivante</t>
+          <t>il roule | roule | avec le chariot | les roues | le chariot | sur les roues | le bol roule</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1421,7 +1431,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Elle fait une chose, puis la suivante. Comment se prépare Nina ?</t>
+          <t>Le bol est trop chaud à porter. Comment avance-t-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1459,7 +1469,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1467,10 +1477,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1485,34 +1495,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>bol</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1521,13 +1535,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1537,13 +1551,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_bol_avance_quand_les_roues_touchent; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
           <t>narrateur|Nina veut le chocolat.
-narrateur|Comment se prépare-t-elle ?</t>
+narrateur|Comment le bol avance-t-il ?</t>
         </is>
       </c>
     </row>
@@ -1570,17 +1584,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Le pull brun est sur la chaise. Nina enfile le pull. Le pull est chaud, un peu lourd. C'est fait. Les chaussettes, ensuite. Nina prend une chaussette du radiateur. Elle est tiède encore. Elle enfile une, puis l'autre. Tu as les pieds au chaud ? Oui, maman. La casserole a fini. On va au bol. Nina marche vers la cuisine. Le carrelage n'est plus froid, avec les chaussettes. Merci, Nina.</t>
+          <t>Nina recule d'un pas. Le carrelage pique. Il brûle, papa. Le chariot est là. Nina regarde le petit chariot. Ses roues touchent le sol. Je ne le porte pas. Elle ouvre les mains. Elle refuse de foncer. Tes pieds, Nina ? Ils sont froids. Elle revient vers le radiateur. La chaussette brune est tiède. Elle enfile une, puis l'autre. Tu as les pieds au chaud ? Oui, maman. Le pull brun attend sur la chaise. Toi aussi. Elle enfile le pull. Le pull est lourd, un peu chaud. Le bol, Nina ? Sur le chariot. Maman verse le cacao. Ça fait un petit chuchotis. Une vapeur monte du bord. Sur la casserole, l'éclat de casserole brille. Je te vois. Nina pose le bol sur le bois. Le chariot tient le bol. Roule. Elle pousse trop fort. Le bol penche. Oh. Elle s'arrête. Une goutte tremble au bord. Elle donne une petite poussée. Les roues tournent. Toc. Le chariot avance. Il roule ! Merci, Nina. Tu le vois, toi ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Le pull brun est sur la chaise. Nina enfile le pull. Le pull est chaud, un peu lourd. C'est fait. Les chaussettes, ensuite. Nina prend une chaussette du radiateur. Elle est tiède encore. Elle enfile une, puis l'autre. Tu as les pieds au chaud ? Oui, maman. La casserole a fini. On va au bol. Nina marche vers la cuisine. Le carrelage n'est plus froid, avec les chaussettes. Merci, Nina.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina recule d'un pas. Le carrelage pique. Il brûle, papa. Le &lt;emphasis level="moderate"&gt;chariot&lt;/emphasis&gt; est là. Nina regarde le petit chariot. Ses roues touchent le sol. Je ne le porte pas. Elle ouvre les mains. Elle refuse de foncer. Tes pieds, Nina ? Ils sont froids. Elle revient vers le radiateur. La chaussette brune est tiède. Elle enfile une, puis l'autre. Tu as les pieds au chaud ? Oui, maman. Le pull brun attend sur la chaise. Toi aussi. Elle enfile le pull. Le pull est lourd, un peu chaud. Le bol, Nina ? Sur le chariot. Maman verse le cacao. Ça fait un petit chuchotis. Une vapeur monte du bord. Sur la casserole, l'éclat de casserole brille. Je te vois. Nina pose le bol sur le bois. Le chariot tient le bol. Roule. Elle pousse trop fort. Le bol penche. Oh. Elle s'arrête. Une goutte tremble au bord. Elle donne une petite poussée. Les roues tournent. Toc. Le chariot avance. Il roule ! Merci, Nina. Tu le vois, toi ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Fabrice a fait l'étape dite. Se lever. S'habiller. Déje&lt;emphasis&gt;une&lt;/emphasis&gt;r. Le sac. Une étape après l'autre.&lt;/slow&gt; [pause]</t>
+          <t>Nina recule d'un pas. Le carrelage pique. Il brûle, papa. Le &lt;emphasis&gt;chariot&lt;/emphasis&gt; est là. Nina regarde le petit chariot. Ses roues touchent le sol. Je ne le porte pas. Elle ouvre les mains. Elle refuse de foncer. Tes pieds, Nina ? Ils sont froids. Elle revient vers le radiateur. La chaussette brune est tiède. Elle enfile une, puis l'autre. Tu as les pieds au chaud ? Oui, maman. Le pull brun attend sur la chaise. Toi aussi. Elle enfile le pull. Le pull est lourd, un peu chaud. Le bol, Nina ? Sur le chariot. Maman verse le cacao. Ça fait un petit chuchotis. Une vapeur monte du bord. Sur la casserole, l'éclat de casserole brille. Je te vois. Nina pose le bol sur le bois. Le chariot tient le bol. Roule. Elle pousse trop fort. Le bol penche. Oh. Elle s'arrête. Une goutte tremble au bord. Elle donne une petite poussée. Les roues tournent. Toc. Le chariot avance. Il roule ! Merci, Nina. Tu le vois, toi ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1627,7 +1641,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1635,10 +1649,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1661,30 +1675,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>chariot</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1693,10 +1707,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1705,30 +1719,63 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_pose_le_bol_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Le pull brun est sur la chaise.
-narrateur|Nina enfile le pull.
-narrateur|Le pull est chaud, un peu lourd.
-enfant-f|C'est fait.
-papa|Les chaussettes, ensuite.
-narrateur|Nina prend une chaussette du radiateur.
-narrateur|Elle est tiède encore.
+          <t>narrateur|Nina recule d'un pas.
+narrateur|Le carrelage pique.
+enfant-f|Il brûle, papa.
+papa|Le chariot est là.
+narrateur|Nina regarde le petit chariot.
+narrateur|Ses roues touchent le sol.
+enfant-f|Je ne le porte pas.
+narrateur|Elle ouvre les mains.
+narrateur|Elle refuse de foncer.
+maman|Tes pieds, Nina ?
+enfant-f|Ils sont froids.
+narrateur|Elle revient vers le radiateur.
+narrateur|La chaussette brune est tiède.
 narrateur|Elle enfile une, puis l'autre.
 maman|Tu as les pieds au chaud ?
 enfant-f|Oui, maman.
-papa|La casserole a fini.
-maman|On va au bol.
-narrateur|Nina marche vers la cuisine.
-narrateur|Le carrelage n'est plus froid, avec les chaussettes.
-papa|Merci, Nina.</t>
+narrateur|Le pull brun attend sur la chaise.
+enfant-f|Toi aussi.
+narrateur|Elle enfile le pull.
+narrateur|Le pull est lourd, un peu chaud.
+papa|Le bol, Nina ?
+enfant-f|Sur le chariot.
+narrateur|Maman verse le cacao.
+narrateur|Ça fait un petit chuchotis.
+narrateur|Une vapeur monte du bord.
+narrateur|Sur la casserole, l'éclat de casserole brille.
+enfant-f|Je te vois.
+narrateur|Nina pose le bol sur le bois.
+narrateur|Le chariot tient le bol.
+enfant-f|Roule.
+narrateur|Elle pousse trop fort.
+narrateur|Le bol penche.
+enfant-f|Oh.
+narrateur|Elle s'arrête.
+narrateur|Une goutte tremble au bord.
+narrateur|Elle donne une petite poussée.
+narrateur|Les roues tournent.
+narrateur|Toc.
+narrateur|Le chariot avance.
+enfant-f|Il roule !
+papa|Merci, Nina.
+maman|Tu le vois, toi ?
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>cacao,roue</t>
         </is>
       </c>
     </row>
@@ -1755,17 +1802,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman verse le cacao. Ça fait un petit chuchotis dans le bol. Une vapeur monte encore. Tu souffles ? Oui. Nina souffle. La vapeur danse, puis s'en va. Tu goûtes ? Il est chaud. Encore un peu. Nina souffle encore. Elle boit une gorgée. Le cacao est doux, un peu sucré. C'est bon. Tu as une moustache. Une ligne brune reste sur la lèvre. Je la garde. Oui, un moment. La casserole ne chante plus. Le sac, après le bol ? Oui. Nina pose le bol vide. Le fond est encore un peu chaud. Les chaussettes brunes restent tièdes. Le radiateur fait un petit bruit. Tu as attendu le bol ? Oui, une chose, puis l'autre. Une bulle éclate encore dans la casserole. Le sucre sent encore, tout bas. Tu as soufflé assez ? Oui, maintenant il est bon.</t>
+          <t>Jusqu'au radiateur ? Oui, papa. Le chariot roule vers la chambre. Une chaussette barre le passage. La roue s'arrête contre le tissu. Je le porte ! Elle saisit le bol trop vite. Le cacao tremble au bord. Oh. Nina s'arrête. Ses mains se ferment, puis s'ouvrent. Elle refuse de foncer. Le bol revient sur le bois. Elle écarte la chaussette du pied. Le passage est libre, un peu sombre. Roule. Le chariot avance. Toc. Les roues frottent le tapis. Ça fait un petit bruit. L'éclat de casserole tremble, puis tient. Il a passé la chaussette. Le radiateur est près du lit. J'y vais. Nina marche à côté, sans le porter. Le bois continue son petit bruit.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman verse le cacao. Ça fait un petit chuchotis dans le bol. Une vapeur monte encore. Tu souffles ? Oui. Nina souffle. La vapeur danse, puis s'en va. Tu goûtes ? Il est chaud. Encore un peu. Nina souffle encore. Elle boit une gorgée. Le cacao est doux, un peu sucré. C'est bon. Tu as une moustache. Une ligne brune reste sur la lèvre. Je la garde. Oui, un moment. La casserole ne chante plus. Le sac, après le bol ? Oui. Nina pose le bol vide. Le fond est encore un peu chaud. Les chaussettes brunes restent tièdes. Le radiateur fait un petit bruit. Tu as attendu le bol ? Oui, une chose, puis l'autre. Une bulle éclate encore dans la casserole. Le sucre sent encore, tout bas. Tu as soufflé assez ? Oui, maintenant il est bon.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Jusqu'au radiateur ? Oui, papa. Le chariot roule vers la chambre. Une &lt;emphasis level="moderate"&gt;chaussette&lt;/emphasis&gt; barre le passage. La roue s'arrête contre le tissu. Je le porte ! Elle saisit le bol trop vite. Le cacao tremble au bord. Oh. Nina s'arrête. Ses mains se ferment, puis s'ouvrent. Elle refuse de foncer. Le bol revient sur le bois. Elle écarte la chaussette du pied. Le passage est libre, un peu sombre. Roule. Le chariot avance. Toc. Les roues frottent le tapis. Ça fait un petit bruit. L'éclat de casserole tremble, puis tient. Il a passé la chaussette. Le radiateur est près du lit. J'y vais. Nina marche à côté, sans le porter. Le bois continue son petit bruit.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Fabrice met les chaussures. Maman ouvre la porte. L'air sent le matin.&lt;/slow&gt; [pause]</t>
+          <t>Jusqu'au radiateur ? Oui, papa. Le chariot roule vers la chambre. Une &lt;emphasis&gt;chaussette&lt;/emphasis&gt; barre le passage. La roue s'arrête contre le tissu. Je le porte ! Elle saisit le bol trop vite. Le cacao tremble au bord. Oh. Nina s'arrête. Ses mains se ferment, puis s'ouvrent. Elle refuse de foncer. Le bol revient sur le bois. Elle écarte la chaussette du pied. Le passage est libre, un peu sombre. Roule. Le chariot avance. Toc. Les roues frottent le tapis. Ça fait un petit bruit. L'éclat de casserole tremble, puis tient. Il a passé la chaussette. Le radiateur est près du lit. J'y vais. Nina marche à côté, sans le porter. Le bois continue son petit bruit. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1812,7 +1859,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1820,10 +1867,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1844,28 +1891,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>chaussette</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1874,10 +1925,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1886,47 +1937,46 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_porter_le_bol; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman verse le cacao.
-narrateur|Ça fait un petit chuchotis dans le bol.
-narrateur|Une vapeur monte encore.
-maman|Tu souffles ?
-enfant-f|Oui.
-narrateur|Nina souffle.
-narrateur|La vapeur danse, puis s'en va.
-papa|Tu goûtes ?
-enfant-f|Il est chaud.
-maman|Encore un peu.
-narrateur|Nina souffle encore.
-narrateur|Elle boit une gorgée.
-narrateur|Le cacao est doux, un peu sucré.
-enfant-f|C'est bon.
-papa|Tu as une moustache.
-narrateur|Une ligne brune reste sur la lèvre.
-enfant-f|Je la garde.
-maman|Oui, un moment.
-narrateur|La casserole ne chante plus.
-papa|Le sac, après le bol ?
-enfant-f|Oui.
-narrateur|Nina pose le bol vide.
-narrateur|Le fond est encore un peu chaud.
-narrateur|Les chaussettes brunes restent tièdes.
-narrateur|Le radiateur fait un petit bruit.
-papa|Tu as attendu le bol ?
-enfant-f|Oui, une chose, puis l'autre.
-narrateur|Une bulle éclate encore dans la casserole.
-narrateur|Le sucre sent encore, tout bas.
-maman|Tu as soufflé assez ?
-enfant-f|Oui, maintenant il est bon.</t>
+          <t>papa|Jusqu'au radiateur ?
+enfant-f|Oui, papa.
+narrateur|Le chariot roule vers la chambre.
+narrateur|Une chaussette barre le passage.
+narrateur|La roue s'arrête contre le tissu.
+enfant-f|Je le porte !
+narrateur|Elle saisit le bol trop vite.
+narrateur|Le cacao tremble au bord.
+enfant-f|Oh.
+narrateur|Nina s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Elle refuse de foncer.
+narrateur|Le bol revient sur le bois.
+narrateur|Elle écarte la chaussette du pied.
+narrateur|Le passage est libre, un peu sombre.
+enfant-f|Roule.
+narrateur|Le chariot avance.
+narrateur|Toc.
+narrateur|Les roues frottent le tapis.
+narrateur|Ça fait un petit bruit.
+narrateur|L'éclat de casserole tremble, puis tient.
+papa|Il a passé la chaussette.
+maman|Le radiateur est près du lit.
+enfant-f|J'y vais.
+narrateur|Nina marche à côté, sans le porter.
+narrateur|Le bois continue son petit bruit.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>porte</t>
+          <t>chaussette,roue</t>
         </is>
       </c>
     </row>
@@ -1953,17 +2003,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai une moustache. Une chose, puis la suivante. Le chocolat est arrivé jusqu'à toi. La vapeur n'est plus sous la porte. Bravo, Nina. La moustache brune reste tiède sur sa lèvre.</t>
+          <t>Ils s'arrêtent près du radiateur. Le métal chante plus loin, faible. Il a fait tout le chemin. Toi aussi. Le bol est chaud, sous ses doigts. Les chaussettes sont chaudes. Tu souffles ? Oui, maman. Nina souffle. La vapeur danse, puis s'en va. Elle boit une gorgée. Le cacao est doux, un peu sucré. C'est bon. Tu as une moustache. Une ligne brune reste sur la lèvre. Je la garde. On est bien, ici. La vapeur n'est plus sous la porte. L'éclat de casserole tient sur le bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai une moustache. Une chose, puis la suivante. Le chocolat est arrivé jusqu'à toi. La vapeur n'est plus sous la porte. Bravo, Nina. La moustache brune reste tiède sur sa lèvre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'arrêtent près du radiateur. Le métal chante plus loin, faible. Il a fait tout le chemin. Toi aussi. Le bol est chaud, sous ses doigts. Les chaussettes sont chaudes. Tu souffles ? Oui, maman. Nina souffle. La vapeur danse, puis s'en va. Elle boit une gorgée. Le cacao est doux, un peu sucré. C'est bon. Tu as une moustache. Une ligne brune reste sur la lèvre. Je la garde. On est bien, ici. La vapeur n'est plus sous la porte. L'&lt;emphasis level="moderate"&gt;éclat de casserole&lt;/emphasis&gt; tient sur le bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'arrêtent près du radiateur. Le métal chante plus loin, faible. Il a fait tout le chemin. Toi aussi. Le bol est chaud, sous ses doigts. Les chaussettes sont chaudes. Tu souffles ? Oui, maman. Nina souffle. La vapeur danse, puis s'en va. Elle boit une gorgée. Le cacao est doux, un peu sucré. C'est bon. Tu as une moustache. Une ligne brune reste sur la lèvre. Je la garde. On est bien, ici. La vapeur n'est plus sous la porte. L'&lt;emphasis&gt;éclat de casserole&lt;/emphasis&gt; tient sur le bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2010,18 +2060,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2030,12 +2080,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2044,17 +2094,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de casserole</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2063,11 +2117,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2076,29 +2130,51 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bord; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai une moustache.
-papa|Une chose, puis la suivante.
-maman|Le chocolat est arrivé jusqu'à toi.
+          <t>narrateur|Ils s'arrêtent près du radiateur.
+narrateur|Le métal chante plus loin, faible.
+enfant-f|Il a fait tout le chemin.
+papa|Toi aussi.
+narrateur|Le bol est chaud, sous ses doigts.
+narrateur|Les chaussettes sont chaudes.
+maman|Tu souffles ?
+enfant-f|Oui, maman.
+narrateur|Nina souffle.
+narrateur|La vapeur danse, puis s'en va.
+narrateur|Elle boit une gorgée.
+narrateur|Le cacao est doux, un peu sucré.
+enfant-f|C'est bon.
+papa|Tu as une moustache.
+narrateur|Une ligne brune reste sur la lèvre.
+enfant-f|Je la garde.
+maman|On est bien, ici.
 narrateur|La vapeur n'est plus sous la porte.
-maman|Bravo, Nina.
-narrateur|La moustache brune reste tiède sur sa lèvre.</t>
+narrateur|L'éclat de casserole tient sur le bord.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>radiateur</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2211,6 +2287,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>